<commit_message>
Add per-trial boat values and fix the speed units
The boat speeds and accelerations are in body lengths per second (and per
second squared), as in Fig. 3. The sheet per_trial of Data_Fig_S25_D,E.xlsx
gives the values of each trial.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data_Fig_03_R,S,T.xlsx
+++ b/Data_Fig_03_R,S,T.xlsx
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Speed_m_s</t>
+          <t>Speed_BL_s</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -434,7 +434,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Acceleration_m_s2</t>
+          <t>Acceleration_BL_s2</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">

</xml_diff>